<commit_message>
fix(apartaderos): validación ADIF con datos reales del BPA (consulta directa)
Códigos/precios verificados en bpa.adif.es:
- Comprobador de aguja = CFA040$ €4.963,85/ud (antes sin código).
- Motor = CFA010$ €10.625 (CORRIGE CBB010, que en BPA es bastidor enclavamiento).
- Desvío = VEA010$ €104.566 (suministro, tipo C r318); señal CCA040$ €7.934.
- ADIF usa GSM-R, no TETRA → terminales TETRA por mercado (confirmado).
- Distinción abatible/no abatible existe en CCA040$ pero solo aplica a ENCE.
Excel: nueva hoja "Validación ADIF". Cifras del modelo sin cambio (orden de magnitud).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IX_WBS_Planificacion/Costo_Apartaderos_PTC.xlsx
+++ b/IX_WBS_Planificacion/Costo_Apartaderos_PTC.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="1 Apartadero" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="10 Apartaderos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Validación ADIF" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,9 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;M&quot;"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
+    <numFmt numFmtId="166" formatCode="#,##0 &quot;€&quot;"/>
+    <numFmt numFmtId="167" formatCode="#,##0.0 &quot;M&quot;"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -130,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -184,6 +187,21 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1027,4 +1045,258 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>VALIDACIÓN CONTRA ADIF BPA 2026  —  consulta directa (bpa.adif.es)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Conversión 4.796 COP/EUR (TRM 4.400 × 1,09). Precios ADIF = referencia europea, trocha estándar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>EXCLUIDOS — no son alcance del apartadero</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Componente</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Código BPA</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Precio €/ud</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>≈ COP (M)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Por qué se excluye</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Aparato de vía — desvío (suministro)</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="inlineStr">
+        <is>
+          <t>VEA010$ (tipo C·r318·nuevo)</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="n">
+        <v>104566</v>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>501.5</v>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Obra civil/vía. Apartaderos existentes (AT1). Montaje en VEC#.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Motor / accionamiento de aguja</t>
+        </is>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>CFA010$</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="n">
+        <v>10625</v>
+      </c>
+      <c r="D7" s="28" t="n">
+        <v>51</v>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>Autotalonable fuera de ENCE — sin motor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Señal luminosa LED</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="inlineStr">
+        <is>
+          <t>CCA040$ (alta no abatible·3 focos)</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="n">
+        <v>7934</v>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>PTC virtual — sin semáforo lateral. Solo ENCE (WBS 1.5.101).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>INCLUIDOS — equipo CTSC incremental</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Componente</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>$M COP (modelo)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Ancla ADIF / referencia</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Comprobador de aguja (×2) + integración CCO</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>92</v>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>ADIF CFA040$ €4.963,85/ud ≈ $23,8M/u (suministro+montaje). 2 ud ≈ $48M base; resto = SIL-4 vital + integración Back Office.</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="n"/>
+      <c r="E12" s="23" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Terminal de datos TETRA (×2)</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>ADIF no usa TETRA sino GSM-R (TMG010 €2.727). Mercado Hytera/Motorola ~$17,5M/u dato industrial.</t>
+        </is>
+      </c>
+      <c r="D13" s="26" t="n"/>
+      <c r="E13" s="26" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Energía solar autónoma &lt;50W + LiFePO4</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>33</v>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Mercado solar local (~$7.500 USD instalado).</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="n"/>
+      <c r="E14" s="23" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>CORRECCIÓN: el código CBB010 no es el motor — en BPA es 'bastidor equipos de enclavamiento' (contadores de ejes). Motor = CFA010$.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>GSM-R vs TETRA: 'TETRA' da cero resultados en BPA — ADIF usa GSM-R. LFC usa TETRA por doctrina (BCD) -&gt; terminales por mercado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Abatibles: la distinción abatible/no abatible existe en CCA040$ (parámetro BPA), pero solo aplica a señales de ENCE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>El comprobador es la línea más sensible: rango ADIF base ~$23,8M/u &lt;-&gt; versión SIL-4 vital. Confirmar vía RFQ.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="C12:E12"/>
+    <mergeCell ref="A18:E18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(apartaderos): trazabilidad ADIF — fuente, fecha, versión y rutas BPA
- HTML/Excel: marca "versión BPA POR CONFIRMAR" (el 2026 era supuesto no
  verificado) + fecha de consulta (2026-05-23) + fuente bpa.adif.es.
- Hoja "Validación ADIF": añade códigos paramétricos completos (VEA010aba,
  CFA010aaa, CCA040ebaad, CFA040caa) y la ruta/capítulo BPA por ítem.
- Nota de pendiente: capturar versión exacta del BPA y URL directa por ítem.
- Hojas de costo: referencia cruzada a la hoja de validación.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IX_WBS_Planificacion/Costo_Apartaderos_PTC.xlsx
+++ b/IX_WBS_Planificacion/Costo_Apartaderos_PTC.xlsx
@@ -568,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -770,10 +770,18 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Anclas de precio / códigos BPA: ver hoja 'Validación ADIF' (fuente bpa.adif.es · consulta 2026-05-23 · versión BPA por confirmar).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A2:D2"/>
@@ -790,7 +798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1032,12 +1040,20 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Anclas de precio / códigos BPA: ver hoja 'Validación ADIF' (fuente bpa.adif.es · consulta 2026-05-23 · versión BPA por confirmar).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="A17:E17"/>
@@ -1053,27 +1069,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VALIDACIÓN CONTRA ADIF BPA 2026  —  consulta directa (bpa.adif.es)</t>
+          <t>VALIDACIÓN CONTRA ADIF — Banco de Precios (BPA)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Conversión 4.796 COP/EUR (TRM 4.400 × 1,09). Precios ADIF = referencia europea, trocha estándar.</t>
+          <t>Fuente: bpa.adif.es (consulta directa)  ·  Fecha de consulta: 2026-05-23  ·  Versión BPA: POR CONFIRMAR  ·  Conversión 4.796 COP/EUR (TRM 4.400 × 1,09)</t>
         </is>
       </c>
     </row>
@@ -1095,17 +1112,22 @@
           <t>Código BPA</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Ruta BPA (capítulo)</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Precio €/ud</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>≈ COP (M)</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Por qué se excluye</t>
         </is>
@@ -1119,16 +1141,21 @@
       </c>
       <c r="B6" s="23" t="inlineStr">
         <is>
-          <t>VEA010$ (tipo C·r318·nuevo)</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="n">
+          <t>VEA010aba</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>V# › VE# › VEA# (Suministro)</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="n">
         <v>104566</v>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="E6" s="25" t="n">
         <v>501.5</v>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>Obra civil/vía. Apartaderos existentes (AT1). Montaje en VEC#.</t>
         </is>
@@ -1142,16 +1169,21 @@
       </c>
       <c r="B7" s="26" t="inlineStr">
         <is>
-          <t>CFA010$</t>
-        </is>
-      </c>
-      <c r="C7" s="27" t="n">
+          <t>CFA010aaa</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>C# › CF# (Aparatos vía) › CFA#</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="n">
         <v>10625</v>
       </c>
-      <c r="D7" s="28" t="n">
+      <c r="E7" s="28" t="n">
         <v>51</v>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>Autotalonable fuera de ENCE — sin motor.</t>
         </is>
@@ -1165,16 +1197,21 @@
       </c>
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>CCA040$ (alta no abatible·3 focos)</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="n">
+          <t>CCA040ebaad</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>C# › CC# › CCA# (Señales laterales)</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="n">
         <v>7934</v>
       </c>
-      <c r="D8" s="25" t="n">
+      <c r="E8" s="25" t="n">
         <v>38.1</v>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>PTC virtual — sin semáforo lateral. Solo ENCE (WBS 1.5.101).</t>
         </is>
@@ -1195,16 +1232,21 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>$M COP (modelo)</t>
+          <t>$M COP</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Ancla ADIF / referencia</t>
+          <t>Ruta BPA / referencia</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr"/>
       <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Detalle</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -1217,11 +1259,16 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>ADIF CFA040$ €4.963,85/ud ≈ $23,8M/u (suministro+montaje). 2 ud ≈ $48M base; resto = SIL-4 vital + integración Back Office.</t>
+          <t>ADIF CFA040caa · C# › CF# › CFA#</t>
         </is>
       </c>
       <c r="D12" s="23" t="n"/>
       <c r="E12" s="23" t="n"/>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>€4.963,85/ud ≈ $23,8M/u (suministro+montaje). 2 ud ≈ $48M base; resto = SIL-4 vital + integración Back Office.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -1234,11 +1281,16 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>ADIF no usa TETRA sino GSM-R (TMG010 €2.727). Mercado Hytera/Motorola ~$17,5M/u dato industrial.</t>
+          <t>Mercado (ADIF no tiene TETRA, usa GSM-R)</t>
         </is>
       </c>
       <c r="D13" s="26" t="n"/>
       <c r="E13" s="26" t="n"/>
+      <c r="F13" s="10" t="inlineStr">
+        <is>
+          <t>Ref. ADIF GSM-R TMG010a €2.727 (terminal mano). Mercado Hytera/Motorola ~$17,5M/u dato industrial.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -1251,11 +1303,16 @@
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>Mercado solar local (~$7.500 USD instalado).</t>
+          <t>Mercado solar local</t>
         </is>
       </c>
       <c r="D14" s="23" t="n"/>
       <c r="E14" s="23" t="n"/>
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>~$7.500 USD instalado.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="19" t="inlineStr">
@@ -1285,17 +1342,25 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>PENDIENTE: capturar la VERSIÓN/año exacta del BPA y la URL directa por ítem en la próxima consulta (no se registraron).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
     <mergeCell ref="C14:E14"/>
-    <mergeCell ref="A17:E17"/>
     <mergeCell ref="C13:E13"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A20:F20"/>
     <mergeCell ref="C12:E12"/>
-    <mergeCell ref="A18:E18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(apartaderos): desglose del comprobador + columna Referencia/Fuente
Transparencia ante Interventoría (evita comparar €5.000 TCO vs $92M opaco):
- Comprobador CTC/PTC desglosado en 3 sublíneas en Excel y HTML:
  hardware $48M (ADIF CFA040$ €4.963,85/u) + cert. SIL-4 $20M + integración $24M
  = $92M (×10: 480/200/240 = $920M). Totales sin cambio.
- Excel: nueva columna "Referencia / Fuente" por línea (ADIF real donde existe,
  GSM-R/mercado y "RFQ pendiente" donde no; FRA/AREMA en servicios).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IX_WBS_Planificacion/Costo_Apartaderos_PTC.xlsx
+++ b/IX_WBS_Planificacion/Costo_Apartaderos_PTC.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="166" formatCode="#,##0 &quot;€&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0.0 &quot;M&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="001B2A41"/>
       <sz val="10"/>
     </font>
@@ -57,9 +63,8 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <color rgb="00555555"/>
+      <sz val="8.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -74,7 +79,7 @@
       <sz val="8.5"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +94,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0014304A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3EEDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -133,74 +143,96 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -568,13 +600,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -587,205 +620,269 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corredor La Dorada–Chiriguaná · Contrato APP No. 001 de 2025 · SICC v14.7</t>
+          <t>Corredor La Dorada–Chiriguaná · Contrato APP No. 001 de 2025 · SICC v14.7 · TRM 4.400 · AIU+IVA 1,18</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>TRM (COP/USD):</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>4400</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Factor AIU+IVA:</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>1.18</v>
+          <t>Cubo</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>COP (millones)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Referencia / Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Terminal de datos TETRA ×2 + alta/programación en red</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>7955</v>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>ADIF no tiene TETRA (usa GSM-R, TMG010 €2.727). Mercado Hytera/Motorola — RFQ pendiente</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Cubo</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>COP (millones)</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>USD</t>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>CTC/PTC</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Comprobador de aguja — hardware (suministro+montaje) ×2</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>10909</v>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>ADIF CFA040$ €4.963,85/ud — bpa.adif.es</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Comunicaciones</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Terminal de datos TETRA ×2 + alta/programación en red</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>7955</v>
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>CTC/PTC</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Certificación SIL-4 + documentación safety case</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>4545</v>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>FRA 49 CFR §236.1005 / EN 50126 — estimación</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>CTC/PTC</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Comprobador de aguja SIL-4 ×2 + integración al PTC del CCO</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="n">
-        <v>92</v>
-      </c>
-      <c r="D8" s="12" t="n">
-        <v>20909</v>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Integración Back Office PTC + prueba funcional E2E (del punto)</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>5455</v>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>AREMA C&amp;S Manual §12 — estimación</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Energía</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Solar autónoma &lt;50 W + batería LiFePO4</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="7" t="n">
         <v>7500</v>
       </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>Mercado Colombia solar industrial — RFQ pendiente</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Servicios</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Instalación + prueba in-situ (SAT)</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
+      <c r="C10" s="14" t="n">
         <v>31</v>
       </c>
-      <c r="D10" s="12" t="n">
+      <c r="D10" s="15" t="n">
         <v>7045</v>
       </c>
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>AREMA C&amp;S §12 — rendimientos de campo (estimación)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Ingeniería</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Diseño + config Back Office (prorrateado ÷10)</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="n">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Diseño de detalle + parametrización (prorrateado ÷10)</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
         <v>90</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="7" t="n">
         <v>20455</v>
       </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>FRA §236.1005 — estimación % CAPEX</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Costo directo (all-in)</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n"/>
-      <c r="C12" s="14" t="n">
+      <c r="B12" s="17" t="n"/>
+      <c r="C12" s="18" t="n">
         <v>281</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="19" t="n">
         <v>63864</v>
       </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>Comprobador (3 sublíneas) = subtotal CTC/PTC $92M</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Con AIU + IVA</t>
         </is>
       </c>
-      <c r="B13" s="16" t="n"/>
-      <c r="C13" s="17" t="n">
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="22" t="n">
         <v>331.6</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="23" t="n">
         <v>75359</v>
       </c>
+      <c r="E13" s="21" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>Cifras de orden de magnitud — sujeto a RFQ formal (Frauscher / Siemens / Hytera).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>NO incluye: alargamiento de apartaderos (obra civil) ni infraestructura TETRA del corredor (ya presupuestada).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
-        <is>
-          <t>Un apartadero lleva: comprobador SIL-4 ×2 + terminal TETRA ×2 + solar. Sin motor, sin señales, sin gabinetes.</t>
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>CTC/PTC = comprobador hardware ($48M) + cert. SIL-4 ($20M) + integración ($24M) = $92M.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
-        <is>
-          <t>Anclas de precio / códigos BPA: ver hoja 'Validación ADIF' (fuente bpa.adif.es · consulta 2026-05-23 · versión BPA por confirmar).</t>
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>Anclas de precio / códigos BPA: ver hoja 'Validación ADIF' (fuente bpa.adif.es · consulta 2026-05-23 · versión por confirmar).</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A17:D17"/>
-    <mergeCell ref="A18:D18"/>
-    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A15:E15"/>
     <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A18:E18"/>
     <mergeCell ref="A12:B12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -798,14 +895,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -818,246 +916,328 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Corredor La Dorada–Chiriguaná · Contrato APP No. 001 de 2025 · SICC v14.7 · 10 apartaderos = 20 desvíos</t>
+          <t>Corredor La Dorada–Chiriguaná · APP No. 001 de 2025 · 10 apartaderos = 20 desvíos · TRM 4.400 · AIU+IVA 1,18</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>TRM (COP/USD):</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n">
-        <v>4400</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>AIU+IVA:</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>1.18</v>
+          <t>Cubo</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Cant.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>COP (millones)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Referencia / Fuente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Terminal de datos TETRA + alta (infra TETRA ya presupuestada)</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>350</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>79545</v>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>ADIF usa GSM-R, no TETRA. Mercado Hytera/Motorola — RFQ</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Cubo</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Cant.</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>COP (millones)</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>USD</t>
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>CTC/PTC</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Comprobador de aguja — hardware (suministro+montaje)</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>480</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>109091</v>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>ADIF CFA040$ €4.963,85/ud — bpa.adif.es</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Comunicaciones</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Terminal de datos TETRA + alta (infra TETRA ya presupuestada)</t>
-        </is>
-      </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="n">
-        <v>350</v>
-      </c>
-      <c r="E7" s="9" t="n">
-        <v>79545</v>
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>CTC/PTC</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Certificación SIL-4 + safety case</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>200</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>45455</v>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>FRA §236.1005 / EN 50126 — estimación</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
         <is>
           <t>CTC/PTC</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>Comprobador de aguja SIL-4 + integración CCO</t>
-        </is>
-      </c>
-      <c r="C8" s="21" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="D8" s="11" t="n">
-        <v>920</v>
-      </c>
-      <c r="E8" s="12" t="n">
-        <v>209091</v>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • Integración Back Office + prueba E2E</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>240</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>54545</v>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>AREMA C&amp;S §12 — estimación</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Energía</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Solar autónoma &lt;50 W + LiFePO4</t>
         </is>
       </c>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="6" t="n">
         <v>330</v>
       </c>
-      <c r="E9" s="9" t="n">
+      <c r="E9" s="7" t="n">
         <v>75000</v>
       </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>Mercado Colombia solar industrial — RFQ</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Servicios de campo</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Instalación + prueba in-situ (SAT)</t>
         </is>
       </c>
-      <c r="C10" s="21" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="D10" s="11" t="n">
+      <c r="D10" s="14" t="n">
         <v>310</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="15" t="n">
         <v>70455</v>
       </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>AREMA C&amp;S §12 — rendimientos de campo</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Ingeniería</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>Diseño + config Back Office (global, una sola vez)</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="6" t="n">
         <v>900</v>
       </c>
-      <c r="E11" s="9" t="n">
+      <c r="E11" s="7" t="n">
         <v>204545</v>
       </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>FRA §236.1005 — estimación % CAPEX</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Costo directo total</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n"/>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="14" t="n">
+      <c r="B12" s="17" t="n"/>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="18" t="n">
         <v>2810</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="E12" s="19" t="n">
         <v>638636</v>
       </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>Comprobador (3 sublíneas) = $920M</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Con AIU + IVA</t>
         </is>
       </c>
-      <c r="B13" s="16" t="n"/>
-      <c r="C13" s="16" t="n"/>
-      <c r="D13" s="17" t="n">
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="21" t="n"/>
+      <c r="D13" s="22" t="n">
         <v>3315.8</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="23" t="n">
         <v>753591</v>
       </c>
+      <c r="F13" s="21" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>Cifras de orden de magnitud — sujeto a RFQ formal (Frauscher / Siemens / Hytera).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>NO incluye: alargamiento de apartaderos (obra civil) ni infraestructura TETRA del corredor (ya presupuestada en el proyecto).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>CTC/PTC = comprobador hardware ($480M) + cert. SIL-4 ($200M) + integración ($240M) = $920M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="inlineStr">
         <is>
           <t>Infraestructura TETRA verificada en WBS v3.0: no hay partida de terminales para apartaderos → el terminal del switch es incremental (sin doble conteo).</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>El costo unitario baja con el volumen: la ingeniería fija (~$900M) se reparte entre más apartaderos.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="19" t="inlineStr">
-        <is>
-          <t>Anclas de precio / códigos BPA: ver hoja 'Validación ADIF' (fuente bpa.adif.es · consulta 2026-05-23 · versión BPA por confirmar).</t>
+    <row r="20">
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>Anclas de precio / códigos BPA: ver hoja 'Validación ADIF' (fuente bpa.adif.es · consulta 2026-05-23 · versión por confirmar).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A18:E18"/>
+    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A15:F15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1095,255 +1275,255 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="22" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>EXCLUIDOS — no son alcance del apartadero</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Componente</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Código BPA</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Ruta BPA (capítulo)</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Precio €/ud</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>≈ COP (M)</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Por qué se excluye</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Aparato de vía — desvío (suministro)</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
         <is>
           <t>VEA010aba</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>V# › VE# › VEA# (Suministro)</t>
         </is>
       </c>
-      <c r="D6" s="24" t="n">
+      <c r="D6" s="30" t="n">
         <v>104566</v>
       </c>
-      <c r="E6" s="25" t="n">
+      <c r="E6" s="31" t="n">
         <v>501.5</v>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>Obra civil/vía. Apartaderos existentes (AT1). Montaje en VEC#.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>Motor / accionamiento de aguja</t>
         </is>
       </c>
-      <c r="B7" s="26" t="inlineStr">
+      <c r="B7" s="32" t="inlineStr">
         <is>
           <t>CFA010aaa</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>C# › CF# (Aparatos vía) › CFA#</t>
         </is>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D7" s="33" t="n">
         <v>10625</v>
       </c>
-      <c r="E7" s="28" t="n">
+      <c r="E7" s="34" t="n">
         <v>51</v>
       </c>
-      <c r="F7" s="10" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>Autotalonable fuera de ENCE — sin motor.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Señal luminosa LED</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
         <is>
           <t>CCA040ebaad</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>C# › CC# › CCA# (Señales laterales)</t>
         </is>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="30" t="n">
         <v>7934</v>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="E8" s="31" t="n">
         <v>38.1</v>
       </c>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="F8" s="5" t="inlineStr">
         <is>
           <t>PTC virtual — sin semáforo lateral. Solo ENCE (WBS 1.5.101).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>INCLUIDOS — equipo CTSC incremental</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Componente</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>$M COP</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Ruta BPA / referencia</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr"/>
-      <c r="E11" s="5" t="inlineStr"/>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Detalle</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Comprobador de aguja (×2) + integración CCO</t>
         </is>
       </c>
-      <c r="B12" s="8" t="n">
+      <c r="B12" s="6" t="n">
         <v>92</v>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>ADIF CFA040caa · C# › CF# › CFA#</t>
         </is>
       </c>
-      <c r="D12" s="23" t="n"/>
-      <c r="E12" s="23" t="n"/>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="D12" s="29" t="n"/>
+      <c r="E12" s="29" t="n"/>
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>€4.963,85/ud ≈ $23,8M/u (suministro+montaje). 2 ud ≈ $48M base; resto = SIL-4 vital + integración Back Office.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Terminal de datos TETRA (×2)</t>
         </is>
       </c>
-      <c r="B13" s="11" t="n">
+      <c r="B13" s="14" t="n">
         <v>35</v>
       </c>
-      <c r="C13" s="10" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>Mercado (ADIF no tiene TETRA, usa GSM-R)</t>
         </is>
       </c>
-      <c r="D13" s="26" t="n"/>
-      <c r="E13" s="26" t="n"/>
-      <c r="F13" s="10" t="inlineStr">
+      <c r="D13" s="32" t="n"/>
+      <c r="E13" s="32" t="n"/>
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>Ref. ADIF GSM-R TMG010a €2.727 (terminal mano). Mercado Hytera/Motorola ~$17,5M/u dato industrial.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Energía solar autónoma &lt;50W + LiFePO4</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>Mercado solar local</t>
         </is>
       </c>
-      <c r="D14" s="23" t="n"/>
-      <c r="E14" s="23" t="n"/>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="29" t="n"/>
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>~$7.500 USD instalado.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>CORRECCIÓN: el código CBB010 no es el motor — en BPA es 'bastidor equipos de enclavamiento' (contadores de ejes). Motor = CFA010$.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>GSM-R vs TETRA: 'TETRA' da cero resultados en BPA — ADIF usa GSM-R. LFC usa TETRA por doctrina (BCD) -&gt; terminales por mercado.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="24" t="inlineStr">
         <is>
           <t>Abatibles: la distinción abatible/no abatible existe en CCA040$ (parámetro BPA), pero solo aplica a señales de ENCE.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="inlineStr">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>El comprobador es la línea más sensible: rango ADIF base ~$23,8M/u &lt;-&gt; versión SIL-4 vital. Confirmar vía RFQ.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>PENDIENTE: capturar la VERSIÓN/año exacta del BPA y la URL directa por ítem en la próxima consulta (no se registraron).</t>
         </is>

</xml_diff>

<commit_message>
docs(apartaderos): BPA versión confirmada (19/02/2026 v1.4.0) + URLs + catálogo
- Versión BPA confirmada: válida desde 19/02/2026, app v1.4.0, bpa.adif.es/bp1;
  precios con costes indirectos 6%. Quitado "versión por confirmar / pendiente".
- Códigos BPA ahora enlazan a su ficha (URLs /concept/...) en HTML.
- Excel: nueva hoja "Referencia BPA" — catálogo de 17 ítems consultados
  (código, precio €, ud, URL, estado): desvío, cerrojo, motor, comprobador,
  señal, UCP ENCE, contador ejes, circuito vía, armario, caja, caseta, SAI,
  cable FO, cable señalización.
- Correcciones: UCP ENCE CAC020$ €118.006 (no €356.780 = sistema completo);
  desvío talonable NO existe en BPA (precio contradictorio).
Cifras del modelo sin cambio.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IX_WBS_Planificacion/Costo_Apartaderos_PTC.xlsx
+++ b/IX_WBS_Planificacion/Costo_Apartaderos_PTC.xlsx
@@ -10,6 +10,7 @@
     <sheet name="1 Apartadero" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="10 Apartaderos" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Validación ADIF" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Referencia BPA" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,13 +19,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;M&quot;"/>
     <numFmt numFmtId="165" formatCode="$#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0 &quot;€&quot;"/>
     <numFmt numFmtId="167" formatCode="#,##0.0 &quot;M&quot;"/>
+    <numFmt numFmtId="168" formatCode="#,##0.00 &quot;€&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,6 +79,12 @@
       <i val="1"/>
       <color rgb="00555555"/>
       <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001155CC"/>
+      <sz val="9"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="8">
@@ -143,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -234,6 +242,30 @@
     </xf>
     <xf numFmtId="167" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1249,7 +1281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1270,7 +1302,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fuente: bpa.adif.es (consulta directa)  ·  Fecha de consulta: 2026-05-23  ·  Versión BPA: POR CONFIRMAR  ·  Conversión 4.796 COP/EUR (TRM 4.400 × 1,09)</t>
+          <t>Fuente: bpa.adif.es/bp1 (app v1.4.0) · BPA válida desde 19/02/2026 · Consulta: 2026-05-23 · Precios con costes indirectos 6% · Conversión 4.796 COP/EUR (TRM 4.400 × 1,09). Detalle y URLs en hoja 'Referencia BPA'.</t>
         </is>
       </c>
     </row>
@@ -1504,33 +1536,40 @@
     <row r="17">
       <c r="A17" s="24" t="inlineStr">
         <is>
-          <t>GSM-R vs TETRA: 'TETRA' da cero resultados en BPA — ADIF usa GSM-R. LFC usa TETRA por doctrina (BCD) -&gt; terminales por mercado.</t>
+          <t>CORRECCIÓN ENCE (no apartadero): la UCP del enclavamiento es CAC020$ €118.006 — la referencia previa de €356.780 era el sistema ENCE completo (módulos CAC010–CAC090).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="24" t="inlineStr">
         <is>
-          <t>Abatibles: la distinción abatible/no abatible existe en CCA040$ (parámetro BPA), pero solo aplica a señales de ENCE.</t>
+          <t>GSM-R vs TETRA: 'TETRA' da cero resultados en BPA — ADIF usa GSM-R. LFC usa TETRA por doctrina (BCD) -&gt; terminales por mercado.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="24" t="inlineStr">
         <is>
-          <t>El comprobador es la línea más sensible: rango ADIF base ~$23,8M/u &lt;-&gt; versión SIL-4 vital. Confirmar vía RFQ.</t>
+          <t>Abatibles: la distinción abatible/no abatible existe en CCA040$ (parámetro BPA), pero solo aplica a señales de ENCE.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="24" t="inlineStr">
         <is>
-          <t>PENDIENTE: capturar la VERSIÓN/año exacta del BPA y la URL directa por ítem en la próxima consulta (no se registraron).</t>
+          <t>El comprobador es la línea más sensible: rango ADIF base ~$23,8M/u &lt;-&gt; versión SIL-4 vital. Confirmar vía RFQ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>Desvío talonable/autotalonable: NO existe partida en BPA (solo tipos C/P/G/AV/B). Requiere precio contradictorio.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="C14:E14"/>
@@ -1540,8 +1579,628 @@
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="C12:E12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>REFERENCIA BPA ADIF — catálogo de ítems consultados</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Fuente: bpa.adif.es/bp1 (app v1.4.0) · BPA válida desde 19/02/2026 · Consulta: 2026-05-23 · Precios con costes indirectos 6%. Códigos $ = paramétricos; el sufijo codifica las opciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Código BPA</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Precio €</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Ud</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>URL / Estado</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>V-1</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Desvío tipo C radio 318 nuevo (suministro)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>VEA010aba</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="n">
+        <v>104565.66</v>
+      </c>
+      <c r="E5" s="25" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F5" s="36" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/156706377</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="inlineStr">
+        <is>
+          <t>V-2</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Desvío talonable / autotalonable</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D6" s="37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" s="38" t="inlineStr">
+        <is>
+          <t>NO EXISTE en BPA — precio contradictorio</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="inlineStr">
+        <is>
+          <t>V-3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Cerrojo de uña, sencillo</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>CFA030aaaa</t>
+        </is>
+      </c>
+      <c r="D7" s="35" t="n">
+        <v>2243.08</v>
+      </c>
+      <c r="E7" s="25" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F7" s="36" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/157968266</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="27" t="inlineStr">
+        <is>
+          <t>S-1</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Motor eléctrico de aguja, sencilla</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>CFA010aaa</t>
+        </is>
+      </c>
+      <c r="D8" s="39" t="n">
+        <v>10624.66</v>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F8" s="40" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/153769673</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>S-2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Comprobador eléctrico de agujas</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>CFA040caa</t>
+        </is>
+      </c>
+      <c r="D9" s="35" t="n">
+        <v>4963.85</v>
+      </c>
+      <c r="E9" s="25" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F9" s="36" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/151681024</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="27" t="inlineStr">
+        <is>
+          <t>S-3</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Señal alta LED, no abatible, 3 focos</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>CCA040ebaad</t>
+        </is>
+      </c>
+      <c r="D10" s="39" t="n">
+        <v>7934.23</v>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F10" s="40" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/153988522</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>S-4</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>UCP enclavamiento electrónico (grande)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>CAC020caa</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="n">
+        <v>118006.02</v>
+      </c>
+      <c r="E11" s="25" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F11" s="36" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/152945939</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>S-5</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Sensor de rueda para desvío (cont. ejes)</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>CBB030ca</t>
+        </is>
+      </c>
+      <c r="D12" s="39" t="n">
+        <v>8286.120000000001</v>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F12" s="40" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/157260724</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>S-5b</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Evaluador 8 contadores de ejes</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>CBB040caa</t>
+        </is>
+      </c>
+      <c r="D13" s="35" t="n">
+        <v>13398.59</v>
+      </c>
+      <c r="E13" s="25" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F13" s="36" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/154836682</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>S-6</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Equipo interior circuito de vía AF</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>CBC030caaa</t>
+        </is>
+      </c>
+      <c r="D14" s="39" t="n">
+        <v>7938.04</v>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F14" s="40" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/152228850</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="25" t="inlineStr">
+        <is>
+          <t>A-1</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Armario de señalización grande</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>CDB010caa</t>
+        </is>
+      </c>
+      <c r="D15" s="35" t="n">
+        <v>4151.33</v>
+      </c>
+      <c r="E15" s="25" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F15" s="36" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/155621679</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>A-2</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Caja de terminales 50 bornas</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>CDA010cba</t>
+        </is>
+      </c>
+      <c r="D16" s="39" t="n">
+        <v>1066.04</v>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F16" s="40" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/156383357</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>A-3</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Caseta prefabricada puesto fijo</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>TMI010</t>
+        </is>
+      </c>
+      <c r="D17" s="35" t="n">
+        <v>7180.94</v>
+      </c>
+      <c r="E17" s="25" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F17" s="36" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/category/149855475</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>E-1</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>SAI 1 kVA / 15 min (baterías incl.)</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>COA090ca</t>
+        </is>
+      </c>
+      <c r="D18" s="39" t="n">
+        <v>2115.07</v>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F18" s="40" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/151067858</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="25" t="inlineStr">
+        <is>
+          <t>E-2</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Banco de baterías independiente</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D19" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" s="42" t="inlineStr">
+        <is>
+          <t>NO EXISTE — incluido en SAI (COA0xx)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>T-1</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>Cable FO 48 fibras PKESP, canalización</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>TCJ010bccca</t>
+        </is>
+      </c>
+      <c r="D20" s="39" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F20" s="40" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/158651112</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="25" t="inlineStr">
+        <is>
+          <t>T-2</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Cable señalización 7x4x0.9 CCPSSP</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>CEA030bacad</t>
+        </is>
+      </c>
+      <c r="D21" s="35" t="n">
+        <v>11.67</v>
+      </c>
+      <c r="E21" s="25" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F21" s="36" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/151181595</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="24" t="inlineStr">
+        <is>
+          <t>URLs verificadas en la consulta del 2026-05-23. Códigos con $ = partida paramétrica (el sufijo de letras fija las opciones).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>Para apartaderos PTC Virtual aplican: comprobador (S-2), terminal datos (mercado, no ADIF) y solar. El resto es referencia / ENCE / vía.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A23:F23"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId15"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(ence): baseline real de un ENCE (bottom-up ADIF) + cierre trazabilidad BPA
Baseline_ENCE_ADIF.xlsx (2 hojas):
- "ENCE tipo": BoQ bottom-up con precios ADIF reales (UCP CAC020 + 8 motores
  CFA010 + 8 comprobadores CFA040 + 12 señales CCA040 + 9 contadores ejes CBB030
  + evaluadores + armarios/cajas/caseta + cables + SAI) + 30% ingeniería.
  Total ~€854k = $931k USD = $4,09B COP por ENCE. Núcleo CAC010/030/040/050
  pendiente de BPA (estimado €150k).
- "x5 + comparación": 5 ENCE ~$20,5B COP ($4,65M USD). Confirma Ardanuy ($869k/u)
  y expone que el WBS v3.0 ($800M/ENCE) subestima ~4-5x.
Cantidades = ENCE promedio (Ardanuy ÷ 5), ajustables por estación.

Apartaderos: añadido TMG010a (GSM-R, URL) al catálogo Referencia BPA y © ADIF 2025
a la cita de fuente (HTML + Excel).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IX_WBS_Planificacion/Costo_Apartaderos_PTC.xlsx
+++ b/IX_WBS_Planificacion/Costo_Apartaderos_PTC.xlsx
@@ -1302,7 +1302,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fuente: bpa.adif.es/bp1 (app v1.4.0) · BPA válida desde 19/02/2026 · Consulta: 2026-05-23 · Precios con costes indirectos 6% · Conversión 4.796 COP/EUR (TRM 4.400 × 1,09). Detalle y URLs en hoja 'Referencia BPA'.</t>
+          <t>Fuente: bpa.adif.es/bp1 (app v1.4.0, © ADIF 2025) · BPA válida desde 19/02/2026 · Consulta: 2026-05-23 · Precios con costes indirectos 6% · Conversión 4.796 COP/EUR (TRM 4.400 × 1,09). Detalle y URLs en hoja 'Referencia BPA'.</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1613,7 +1613,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fuente: bpa.adif.es/bp1 (app v1.4.0) · BPA válida desde 19/02/2026 · Consulta: 2026-05-23 · Precios con costes indirectos 6%. Códigos $ = paramétricos; el sufijo codifica las opciones.</t>
+          <t>Fuente: bpa.adif.es/bp1 (app v1.4.0, © ADIF 2025) · BPA válida desde 19/02/2026 · Consulta: 2026-05-23 · Precios con costes indirectos 6%. Códigos $ = paramétricos; el sufijo codifica las opciones.</t>
         </is>
       </c>
     </row>
@@ -2163,15 +2163,45 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="24" t="inlineStr">
-        <is>
-          <t>URLs verificadas en la consulta del 2026-05-23. Códigos con $ = partida paramétrica (el sufijo de letras fija las opciones).</t>
+    <row r="22">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>T-3</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Terminal de mano GSM-R OPS (ADIF no usa TETRA)</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>TMG010a</t>
+        </is>
+      </c>
+      <c r="D22" s="39" t="n">
+        <v>2727.38</v>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>ud</t>
+        </is>
+      </c>
+      <c r="F22" s="40" t="inlineStr">
+        <is>
+          <t>https://bpa.adif.es/bp1/#/concept/158097881</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>URLs verificadas en la consulta del 2026-05-23. Códigos con $ = partida paramétrica (el sufijo de letras fija las opciones).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="24" t="inlineStr">
         <is>
           <t>Para apartaderos PTC Virtual aplican: comprobador (S-2), terminal datos (mercado, no ADIF) y solar. El resto es referencia / ENCE / vía.</t>
         </is>
@@ -2182,7 +2212,7 @@
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
@@ -2200,6 +2230,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>